<commit_message>
Add AOM seat machining clearance to lattice and splitting boards
</commit_message>
<xml_diff>
--- a/Production/LatticeBoardV9/Lattice_Board_V9.xlsx
+++ b/Production/LatticeBoardV9/Lattice_Board_V9.xlsx
@@ -1,131 +1,130 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheets>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R17ea18d8122c4239"/>
+  </x:sheets>
+  <x:definedNames/>
+</x:workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-    </font>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
+<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:fonts count="2">
+    <x:font>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+    </x:font>
+  </x:fonts>
+  <x:fills count="2">
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+  </x:fills>
+  <x:borders count="1">
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+  </x:borders>
+  <x:cellStyleXfs count="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </x:cellStyleXfs>
+  <x:cellXfs count="3">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+  </x:cellXfs>
+  <x:cellStyles count="1">
+    <x:cellStyle name="Normal" xfId="0"/>
+  </x:cellStyles>
+  <x:colors>
+    <x:indexedColors>
+      <x:rgbColor rgb="00000000"/>
+      <x:rgbColor rgb="00FFFFFF"/>
+      <x:rgbColor rgb="00FF0000"/>
+      <x:rgbColor rgb="0000FF00"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00000000"/>
+      <x:rgbColor rgb="00FFFFFF"/>
+      <x:rgbColor rgb="00FF0000"/>
+      <x:rgbColor rgb="0000FF00"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00800000"/>
+      <x:rgbColor rgb="00008000"/>
+      <x:rgbColor rgb="00000080"/>
+      <x:rgbColor rgb="00808000"/>
+      <x:rgbColor rgb="00800080"/>
+      <x:rgbColor rgb="00008080"/>
+      <x:rgbColor rgb="00C0C0C0"/>
+      <x:rgbColor rgb="00808080"/>
+      <x:rgbColor rgb="009999FF"/>
+      <x:rgbColor rgb="00993366"/>
+      <x:rgbColor rgb="00FFFFCC"/>
+      <x:rgbColor rgb="00CCFFFF"/>
+      <x:rgbColor rgb="00660066"/>
+      <x:rgbColor rgb="00FF8080"/>
+      <x:rgbColor rgb="000066CC"/>
+      <x:rgbColor rgb="00CCCCFF"/>
+      <x:rgbColor rgb="00000080"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00800080"/>
+      <x:rgbColor rgb="00800000"/>
+      <x:rgbColor rgb="00008080"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="0000CCFF"/>
+      <x:rgbColor rgb="00CCFFFF"/>
+      <x:rgbColor rgb="00CCFFCC"/>
+      <x:rgbColor rgb="00FFFF99"/>
+      <x:rgbColor rgb="0099CCFF"/>
+      <x:rgbColor rgb="00FF99CC"/>
+      <x:rgbColor rgb="00CC99FF"/>
+      <x:rgbColor rgb="00FFCC99"/>
+      <x:rgbColor rgb="003366FF"/>
+      <x:rgbColor rgb="0033CCCC"/>
+      <x:rgbColor rgb="0099CC00"/>
+      <x:rgbColor rgb="00FFCC00"/>
+      <x:rgbColor rgb="00FF9900"/>
+      <x:rgbColor rgb="00FF6600"/>
+      <x:rgbColor rgb="00666699"/>
+      <x:rgbColor rgb="00969696"/>
+      <x:rgbColor rgb="00003366"/>
+      <x:rgbColor rgb="00339966"/>
+      <x:rgbColor rgb="00003300"/>
+      <x:rgbColor rgb="00333300"/>
+      <x:rgbColor rgb="00993300"/>
+      <x:rgbColor rgb="00993366"/>
+      <x:rgbColor rgb="00333399"/>
+      <x:rgbColor rgb="00333333"/>
+    </x:indexedColors>
+  </x:colors>
+</x:styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -292,7 +291,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -301,13 +300,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -341,17 +340,6 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -406,8 +394,6 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -427,7 +413,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Lattice board V9.7 with cell enclosure V9.16 (24 x 15 in, f = 300 folded cat-eyes, sliding Rb cell enclosure of two identical half bodies, two end screws) - single-TA configuration + external-TA option</t>
+          <t xml:space="preserve">Lattice board V9.7 with cell enclosure V9.16 (24 x 15 in, f = 300 folded cat-eyes, sliding Rb cell enclosure of two identical half bodies, two end screws) - single-TA configuration + external-TA option</t>
         </is>
       </c>
     </row>
@@ -435,19 +421,19 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Adaptors</t>
+          <t xml:space="preserve">Adaptors</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>#</t>
+          <t xml:space="preserve">#</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AOM_Adapter.step (upper AOM adapter; the lower seat is machined into the baseplate)</t>
+          <t xml:space="preserve">AOM_Adapter.step (upper AOM adapter; the lower seat is machined into the baseplate)</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -457,7 +443,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cube_Mount_Halfinch.step</t>
+          <t xml:space="preserve">Cube_Mount_Halfinch.step</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -467,7 +453,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Iris_Mount.step (IDA12 slide mount)</t>
+          <t xml:space="preserve">Iris_Mount.step (IDA12 slide mount)</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -477,7 +463,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rb_Cell_Enclosure_Cover_V9_16.step (Production/CellEnclosure; machined, 7 mm end cover, no aperture yet)</t>
+          <t xml:space="preserve">Rb_Cell_Enclosure_Cover_V9_16.step (Production/CellEnclosure; machined, 7 mm end cover, no aperture yet)</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -487,7 +473,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rb_Cell_Enclosure_HalfBody_V9_16.step (Production/CellEnclosure; machined half body 88 x 46.9 x 24, two plain through slots; lower and upper half are this same part)</t>
+          <t xml:space="preserve">Rb_Cell_Enclosure_HalfBody_V9_16.step (Production/CellEnclosure; machined half body 88 x 46.9 x 24, two plain through slots; lower and upper half are this same part)</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -497,7 +483,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Shutter_Adapter.step</t>
+          <t xml:space="preserve">Shutter_Adapter.step</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -507,7 +493,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Surface_Adapter_isolator_lip.step</t>
+          <t xml:space="preserve">Surface_Adapter_isolator_lip.step</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -517,7 +503,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Surface_Adapter_rsp05_lip.step</t>
+          <t xml:space="preserve">Surface_Adapter_rsp05_lip.step</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -527,7 +513,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TA_adapter.step</t>
+          <t xml:space="preserve">TA_adapter.step</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -537,7 +523,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8-32 UNC x 5/8 in socket head cap screw (8 cover screws of the cell enclosure)</t>
+          <t xml:space="preserve">8-32 UNC x 5/8 in socket head cap screw (8 cover screws of the cell enclosure)</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -547,7 +533,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8-32 UNC x 2-1/4 in socket head cap screw (through the slots of both enclosure halves into the plate, one per end)</t>
+          <t xml:space="preserve">8-32 UNC x 2-1/4 in socket head cap screw (through the slots of both enclosure halves into the plate, one per end)</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -557,7 +543,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>#8 flat washer (under the two 2-1/4 in screw heads, on the slots)</t>
+          <t xml:space="preserve">#8 flat washer (under the two 2-1/4 in screw heads, on the slots)</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -567,7 +553,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Lattice_V9_7_baseplate_24x15in.step</t>
+          <t xml:space="preserve">Lattice_V9_7_baseplate_24x15in.step</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -578,19 +564,19 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>Elements</t>
+          <t xml:space="preserve">Elements</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>#</t>
+          <t xml:space="preserve">#</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1/2 in half-wave waveplate (HWP)</t>
+          <t xml:space="preserve">1/2 in half-wave waveplate (HWP)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -600,7 +586,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1/2 in mirror (BB05-E03 or equivalent)</t>
+          <t xml:space="preserve">1/2 in mirror (BB05-E03 or equivalent)</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -610,7 +596,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1/2 in quarter-wave waveplate (QWP)</t>
+          <t xml:space="preserve">1/2 in quarter-wave waveplate (QWP)</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -620,7 +606,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1/4-20 table bolt (baseplate fixing)</t>
+          <t xml:space="preserve">1/4-20 table bolt (baseplate fixing)</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -630,7 +616,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>C220TMD-A fiber lens</t>
+          <t xml:space="preserve">C220TMD-A fiber lens</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -640,7 +626,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>G&amp;H AOMO 3100-125</t>
+          <t xml:space="preserve">G&amp;H AOMO 3100-125</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -650,7 +636,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HKTS-5/64 thumbscrew adjuster</t>
+          <t xml:space="preserve">HKTS-5/64 thumbscrew adjuster</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -660,7 +646,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>IDA12-P5 iris</t>
+          <t xml:space="preserve">IDA12-P5 iris</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -670,7 +656,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>IOT-5-850-VLP isolator (113.5 mm plate pocket)</t>
+          <t xml:space="preserve">IOT-5-850-VLP isolator (113.5 mm plate pocket)</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -680,7 +666,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>KA05T fiber port mount (rear tail-clamp hole pair drilled in the plate: lattice 76 mm, TA / AOM boards 82.7 mm behind the head)</t>
+          <t xml:space="preserve">KA05T fiber port mount (rear tail-clamp hole pair drilled in the plate: lattice 76 mm, TA / AOM boards 82.7 mm behind the head)</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -690,7 +676,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>KM100PM (bridged)</t>
+          <t xml:space="preserve">KM100PM (bridged)</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -700,7 +686,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Lens LA1289-B</t>
+          <t xml:space="preserve">Lens LA1289-B</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -710,7 +696,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Lens LA1540-B</t>
+          <t xml:space="preserve">Lens LA1540-B</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -720,7 +706,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Lens LA1618-B</t>
+          <t xml:space="preserve">Lens LA1618-B</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -730,7 +716,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Newport M05 mirror mount</t>
+          <t xml:space="preserve">Newport M05 mirror mount</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -740,7 +726,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PBS cube 12.7 mm</t>
+          <t xml:space="preserve">PBS cube 12.7 mm</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -750,7 +736,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>POLARIS-L05G lens holder (no alignment-pin slots cut)</t>
+          <t xml:space="preserve">POLARIS-L05G lens holder (no alignment-pin slots cut)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -760,7 +746,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>RSP05 rotation mount</t>
+          <t xml:space="preserve">RSP05 rotation mount</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -770,7 +756,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Rb vapour cell GC25075-RB (25.4 x 71.84 mm, fill stem sideways in the parting plane, toward board -x)</t>
+          <t xml:space="preserve">Rb vapour cell GC25075-RB (25.4 x 71.84 mm, fill stem sideways in the parting plane, toward board -x)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -780,7 +766,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>S05TM09</t>
+          <t xml:space="preserve">S05TM09</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -790,7 +776,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SM05FCA2</t>
+          <t xml:space="preserve">SM05FCA2</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -800,7 +786,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SM05L05</t>
+          <t xml:space="preserve">SM05L05</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -810,7 +796,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SRS SR475 shutter</t>
+          <t xml:space="preserve">SRS SR475 shutter</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -820,7 +806,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TA butterfly package (TAboard), mounted on the TA adapter</t>
+          <t xml:space="preserve">TA butterfly package (TAboard), mounted on the TA adapter</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -831,19 +817,19 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>External-TA option only (not installed in the single-TA configuration)</t>
+          <t xml:space="preserve">External-TA option only (not installed in the single-TA configuration)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>#</t>
+          <t xml:space="preserve">#</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Iris_Mount.step (IDA12 slide mount)</t>
+          <t xml:space="preserve">Iris_Mount.step (IDA12 slide mount)</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -853,7 +839,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1/2 in mirror (BB05-E03 or equivalent)</t>
+          <t xml:space="preserve">1/2 in mirror (BB05-E03 or equivalent)</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -863,7 +849,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>C220TMD-A fiber lens</t>
+          <t xml:space="preserve">C220TMD-A fiber lens</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -873,7 +859,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>HKTS-5/64 thumbscrew adjuster</t>
+          <t xml:space="preserve">HKTS-5/64 thumbscrew adjuster</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -883,7 +869,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IDA12-P5 iris</t>
+          <t xml:space="preserve">IDA12-P5 iris</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -893,7 +879,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>KA05T fiber port mount (rear tail-clamp hole pair drilled in the plate: lattice 76 mm, TA / AOM boards 82.7 mm behind the head)</t>
+          <t xml:space="preserve">KA05T fiber port mount (rear tail-clamp hole pair drilled in the plate: lattice 76 mm, TA / AOM boards 82.7 mm behind the head)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -903,7 +889,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Newport M05 mirror mount</t>
+          <t xml:space="preserve">Newport M05 mirror mount</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -913,7 +899,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>S05TM09</t>
+          <t xml:space="preserve">S05TM09</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -923,7 +909,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SM05FCA2</t>
+          <t xml:space="preserve">SM05FCA2</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -933,7 +919,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SM05L05</t>
+          <t xml:space="preserve">SM05L05</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -944,84 +930,83 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t xml:space="preserve">Notes</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Which holes are tapped and which are not: see Lattice_V9_7_baseplate_TAP_or_NOT next to the STEP file (100 x 8-32 tapped, 4 x 1/4-20 table-bolt clearance); for the cell enclosure parts see Production/CellEnclosure/Rb_Cell_Enclosure_V9_16_3D_TAP.png.</t>
+          <t xml:space="preserve">Which holes are tapped and which are not: see Lattice_V9_7_baseplate_TAP_or_NOT next to the STEP file (100 x 8-32 tapped, 4 x 1/4-20 table-bolt clearance); for the cell enclosure parts see Production/CellEnclosure/Rb_Cell_Enclosure_V9_16_3D_TAP.png.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Counts come from the FreeCAD model (Lattice_V9_dual_validation.json); adapters are per hana-branch Production/Adapters STEP names.</t>
+          <t xml:space="preserve">Counts come from the FreeCAD model (Lattice_V9_dual_validation.json); adapters are per hana-branch Production/Adapters STEP names.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>The empty RSP05 mounts on the output rows receive a bonded PBS cube each (not modelled): add 1 cube per "empty rotating PBS RSP05".</t>
+          <t xml:space="preserve">The empty RSP05 mounts on the output rows receive a bonded PBS cube each (not modelled): add 1 cube per "empty rotating PBS RSP05".</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>HKTS-5/64 adjusters are the two per M05 / KA05T mount (already included with the mounts if bought as kits). Every mirror on this board is in a Newport M05.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>AOM seats are machined into the baseplate (integral seat, flat screw face); only the upper AOM adapter is a separate part.</t>
-        </is>
-      </c>
+          <t xml:space="preserve">HKTS-5/64 adjusters are the two per M05 / KA05T mount (already included with the mounts if bought as kits). Every mirror on this board is in a Newport M05.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="88" customHeight="1">
+      <c r="A61" s="2" t="str">
+        <v>The 2 integral AOM seats have 6 mm side clearance and a 4 mm-deep front relief with R3 corners. Bearing faces and installation height are unchanged. Only the upper AOM adapter is a separate part. Single-axis pitch-down 0-4 degrees has a minimum floor gap of 1.06559 mm and sidewall gap of 3 mm. Combined-axis travel is not certified. Use the configuration-specific STEP/tapping sheet for f75-50 or f75-75; their original optional mounting recesses differ from f300.</v>
+      </c>
+      <c r="B61" s="2"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Cat-eye lens LA1618-B (f = 300 mm, 1/2 in): catalogue R 155.0 / tc 2.2 / te 2.1 mm. The plate was laid out with R 154.5 / tc 2.0; the resulting 1.2 / 1.0 mm cat-eye defocus is accepted (see the script docstring).</t>
+          <t xml:space="preserve">Cat-eye lens LA1618-B (f = 300 mm, 1/2 in): catalogue R 155.0 / tc 2.2 / te 2.1 mm. The plate was laid out with R 154.5 / tc 2.0; the resulting 1.2 / 1.0 mm cat-eye defocus is accepted (see the script docstring).</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>The TA butterfly board is screwed to the TA adapter (four M2.5 tapped in the adapter); the plate under the TA has only the adapter's four 8-32 taps, no M2.5 holes. Which holes are tapped: see the TAP_or_NOT sheet next to the STEP file.</t>
+          <t xml:space="preserve">The TA butterfly board is screwed to the TA adapter (four M2.5 tapped in the adapter); the plate under the TA has only the adapter's four 8-32 taps, no M2.5 holes. Which holes are tapped: see the TAP_or_NOT sheet next to the STEP file.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Table bolts (V9.4.2): the four 1/4-20 clearance holes sit on the lab table 1 in grid with the plate fiber-side (right) edge 0.25 in inside the table edge; both pairs 10 in apart and centred on the short edge - fiber-side pair 6.25 in from the right plate edge, TA-side pair 1.5 in from the left edge (16 in further left). STEP coordinates (mm): (447.675, 50.8), (447.675, 304.8), (41.275, 50.8), (41.275, 304.8).</t>
+          <t xml:space="preserve">Table bolts (V9.4.2): the four 1/4-20 clearance holes sit on the lab table 1 in grid with the plate fiber-side (right) edge 0.25 in inside the table edge; both pairs 10 in apart and centred on the short edge - fiber-side pair 6.25 in from the right plate edge, TA-side pair 1.5 in from the left edge (16 in further left). STEP coordinates (mm): (447.675, 50.8), (447.675, 304.8), (41.275, 50.8), (41.275, 304.8).</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>OPTIONAL f = 75 mm cat-eye (the V9.3 LA1612-B set) on the 0-order (input) axis straight after each AOM, bare holes only, nothing installed and nothing listed above: per AOM arm one L05G tap, two RSP05 taps, one slide-mount tap and two M05 taps (lens-&gt;mirror 50 and 75). To use it: 1 x LA1612-B in a POLARIS-L05G, 1 x RSP05 + lip adapter with a 1/2 in QWP, 1 x IDA12 on the slide mount, 1 x M05 retro mirror per arm. The M05 at those positions has no thumbscrew pocket: drive its lower adjuster with a plain 5/64 hex key (no HKTS). The lens-&gt;mirror 75 mirror body stands where fold F1 (DP1) / F3 (DP2) is, so that fold comes off for a 75/75 test.</t>
+          <t xml:space="preserve">OPTIONAL f = 75 mm cat-eye (the V9.3 LA1612-B set) on the 0-order (input) axis straight after each AOM, bare holes only, nothing installed and nothing listed above: per AOM arm one L05G tap, two RSP05 taps, one slide-mount tap and two M05 taps (lens-&gt;mirror 50 and 75). To use it: 1 x LA1612-B in a POLARIS-L05G, 1 x RSP05 + lip adapter with a 1/2 in QWP, 1 x IDA12 on the slide mount, 1 x M05 retro mirror per arm. The M05 at those positions has no thumbscrew pocket: drive its lower adjuster with a plain 5/64 hex key (no HKTS). The lens-&gt;mirror 75 mirror body stands where fold F1 (DP1) / F3 (DP2) is, so that fold comes off for a 75/75 test.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Six common stations are drilled as bare 8-32 holes; no holder or optic is installed. They are sized for a POLARIS-L05G with a 10 mm cylindrical lens bonded to its front face.</t>
+          <t xml:space="preserve">Six common stations are drilled as bare 8-32 holes; no holder or optic is installed. They are sized for a POLARIS-L05G with a 10 mm cylindrical lens bonded to its front face.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Cell enclosure V9.16 (the plate and its seat are unchanged since V9.7): the seat is an 11.3 mm deep pocket (104.4 x 64.7 mm, board x 157.8..222.5 / y 111.3..215.7) with two 8-32 taps through its floor at (185, 123.6) and (185, 203.4). The split plain-block enclosure is 2 identical half bodies (the upper one is the lower one turned over) + 2 identical end covers (Production/CellEnclosure). Two 8-32 x 2-1/4 in socket head cap screws with #8 flat washers, one per end, go from the top face through the plain through slots of both halves (in the bore end regions beyond the cell; no counter-slot, the heads sit on the top face) into the taps (9.2 mm of thread in the 14.1 mm pocket floor) and clamp the halves and the position; travel 10.5 mm toward -x (beam through the cell centre .. 2.2 mm inside the cell wall). The end covers (7 mm) are held by 8 x 8-32 x 5/8 in socket head cap screws (counterbored 3.5, 16 mm deep taps, two in each end face of each half) and tie the halves together. The fill stem (Thorlabs 24088-E0W: mid-length, &lt; 10 mm high) lies in the parting plane toward -x in a closed 12 x 10 pocket; the 6 x 6 cable notch is in the middle of the opposite (+x) wall, 3 mm in each half, 9.7..15.7 mm above the plate top. Beam apertures in the covers are not yet machined.</t>
+          <t xml:space="preserve">Cell enclosure V9.16 (the plate and its seat are unchanged since V9.7): the seat is an 11.3 mm deep pocket (104.4 x 64.7 mm, board x 157.8..222.5 / y 111.3..215.7) with two 8-32 taps through its floor at (185, 123.6) and (185, 203.4). The split plain-block enclosure is 2 identical half bodies (the upper one is the lower one turned over) + 2 identical end covers (Production/CellEnclosure). Two 8-32 x 2-1/4 in socket head cap screws with #8 flat washers, one per end, go from the top face through the plain through slots of both halves (in the bore end regions beyond the cell; no counter-slot, the heads sit on the top face) into the taps (9.2 mm of thread in the 14.1 mm pocket floor) and clamp the halves and the position; travel 10.5 mm toward -x (beam through the cell centre .. 2.2 mm inside the cell wall). The end covers (7 mm) are held by 8 x 8-32 x 5/8 in socket head cap screws (counterbored 3.5, 16 mm deep taps, two in each end face of each half) and tie the halves together. The fill stem (Thorlabs 24088-E0W: mid-length, &lt; 10 mm high) lies in the parting plane toward -x in a closed 12 x 10 pocket; the 6 x 6 cable notch is in the middle of the opposite (+x) wall, 3 mm in each half, 9.7..15.7 mm above the plate top. Beam apertures in the covers are not yet machined.</t>
         </is>
       </c>
     </row>

</xml_diff>